<commit_message>
Fix site mapping flow input validation
</commit_message>
<xml_diff>
--- a/docs/week04/HE_Toolkit_dashboard_standard_data_template.xlsx
+++ b/docs/week04/HE_Toolkit_dashboard_standard_data_template.xlsx
@@ -1091,16 +1091,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:T201"/>
-  <dataValidations count="4">
-    <dataValidation sqref="C2:C201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"HDE,NRFA,FLOWFILES,LOCAL"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C2:C5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"HDE,NRFA"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C2:C5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"HDE,NRFA"</formula1>
-    </dataValidation>
+  <dataValidations count="1">
     <dataValidation sqref="G2:G5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"HDE,NRFA"</formula1>
     </dataValidation>

</xml_diff>